<commit_message>
Set workbook spacer rows to 3px equivalent
</commit_message>
<xml_diff>
--- a/Essential55_Paper_Practice_Workbook.xlsx
+++ b/Essential55_Paper_Practice_Workbook.xlsx
@@ -648,7 +648,7 @@
       <c r="J2" s="16" t="n"/>
       <c r="K2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="G3" s="9" t="n"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -2088,7 +2088,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -3528,7 +3528,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -4990,7 +4990,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -5863,7 +5863,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -6430,7 +6430,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -7303,7 +7303,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -7870,7 +7870,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -9081,7 +9081,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -9648,7 +9648,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -10983,7 +10983,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -11550,7 +11550,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -13121,7 +13121,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -13688,7 +13688,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -15331,7 +15331,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -15898,7 +15898,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -17084,7 +17084,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -17651,7 +17651,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -18586,7 +18586,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -19147,7 +19147,7 @@
       <c r="J2" s="16" t="n"/>
       <c r="K2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="G3" s="9" t="n"/>
@@ -20015,7 +20015,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -20582,7 +20582,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -21521,7 +21521,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -22088,7 +22088,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -23269,7 +23269,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -23836,7 +23836,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -25267,7 +25267,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -25834,7 +25834,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -27221,7 +27221,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -27788,7 +27788,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -28963,7 +28963,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -29530,7 +29530,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -30535,7 +30535,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -31102,7 +31102,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -33011,7 +33011,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -33578,7 +33578,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -34871,7 +34871,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -35438,7 +35438,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -37055,7 +37055,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -37622,7 +37622,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -38842,7 +38842,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -39409,7 +39409,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -40282,7 +40282,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -40849,7 +40849,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -42148,7 +42148,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -42715,7 +42715,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -43588,7 +43588,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -44155,7 +44155,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -45050,7 +45050,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -45617,7 +45617,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -46490,7 +46490,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -47057,7 +47057,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -47930,7 +47930,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -48497,7 +48497,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -49370,7 +49370,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
@@ -49937,7 +49937,7 @@
       <c r="K2" s="16" t="n"/>
       <c r="L2" s="17" t="n"/>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="1.8" customHeight="1">
       <c r="B3" s="9" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="H3" s="9" t="n"/>
@@ -50810,7 +50810,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="3" customHeight="1">
+    <row r="35" ht="1.8" customHeight="1">
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>

</xml_diff>

<commit_message>
Fix weekly verb QC highlighting issues
</commit_message>
<xml_diff>
--- a/Essential55_Paper_Practice_Workbook.xlsx
+++ b/Essential55_Paper_Practice_Workbook.xlsx
@@ -3636,7 +3636,29 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>roto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ro</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>t</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -4212,29 +4234,7 @@
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <sz val="11"/>
-            </rPr>
-            <t>l</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <b val="1"/>
-              <color rgb="FFFF00A8"/>
-              <sz val="11"/>
-            </rPr>
-            <t>l</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <sz val="11"/>
-            </rPr>
-            <t>impiará</t>
-          </r>
+          <t>limpiará</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -11653,12 +11653,56 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>puesto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>p</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>uest</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>puesto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>p</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>uest</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -13831,7 +13875,29 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>vuelto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>v</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>uelt</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="H7" s="9" t="n"/>
@@ -19260,7 +19326,29 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>escrito</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>escri</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>t</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="G7" s="9" t="n"/>
@@ -33686,7 +33774,29 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>visto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>vi</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>st</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -35585,12 +35695,56 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>hecho</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ech</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>dicho</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>d</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ich</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -42828,7 +42982,29 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>abierto</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ab</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="FFFF00A8"/>
+              <sz val="11"/>
+            </rPr>
+            <t>iert</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <sz val="11"/>
+            </rPr>
+            <t>o</t>
+          </r>
         </is>
       </c>
       <c r="H7" s="9" t="n"/>
@@ -44263,29 +44439,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <sz val="11"/>
-            </rPr>
-            <t>compren</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <b val="1"/>
-              <color rgb="FFFF00A8"/>
-              <sz val="11"/>
-            </rPr>
-            <t>di</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Aptos Narrow"/>
-              <sz val="11"/>
-            </rPr>
-            <t>do</t>
-          </r>
+          <t>comprendido</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">

</xml_diff>